<commit_message>
feat(recon): surface unmatched income rows in UI and output file
The "N unmatched income rows" notice was vague — no way to see which rows.

- Pipeline now exposes the full unmatched list (unmatched.rows: order id,
  product name, released) instead of a 5-row sample, threaded through the API
  and page to the banner.
- UnmatchedBanner gains a "Show unmatched rows" expander rendering a compact
  table (Order ID / Product Name / Released), collapsed by default.
- Output workbook gains a dedicated "Unmatched" sheet with the same columns, so
  the download is self-explanatory instead of folding unmatched dollars into
  Income Compiled under a blank SKU. Empty sheet = none unmatched.
- Regenerated the UAT output artifacts to include the new sheet.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/uat-artifacts/recon-output-2025-07.xlsx
+++ b/docs/uat-artifacts/recon-output-2025-07.xlsx
@@ -7,13 +7,14 @@
     <sheet sheetId="1" name="Income Compiled" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Product Breakdown" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Income Summary" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Unmatched" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3449" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3452" uniqueCount="301">
   <si>
     <t>SKU Reference No.</t>
   </si>
@@ -18663,4 +18664,31 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>